<commit_message>
Sync planning SharePoint : S36
</commit_message>
<xml_diff>
--- a/Plannings 2026 S36.xlsx
+++ b/Plannings 2026 S36.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{0278C15E-DB9E-420E-BCF6-8D5039F54895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CBF2D94-5381-4C46-8B6F-BA9358BC31BC}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{0278C15E-DB9E-420E-BCF6-8D5039F54895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA87EB17-AAC8-4745-AA2F-A68D30C41B68}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="109">
   <si>
     <t>Planning des salariés du 31/08/2026 au 06/09/2026</t>
   </si>
@@ -4151,6 +4151,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="74" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC1A7834-79AC-44D3-87A1-1E369F5D564C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6817179" y="8450036"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5192,7 +5236,9 @@
         <v>13</v>
       </c>
       <c r="G42" s="18"/>
-      <c r="H42" s="19"/>
+      <c r="H42" s="18" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="43" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="20"/>
@@ -5206,7 +5252,9 @@
         <v>14</v>
       </c>
       <c r="G43" s="21"/>
-      <c r="H43" s="22"/>
+      <c r="H43" s="21" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="17" t="s">
@@ -6255,13 +6303,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F17346FA-F5EE-44FA-A68F-F6F1F5BE0D05}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C61972E5-2584-4F29-8D7A-FAC1D583D6EA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15B4A931-4745-42E2-BFB6-5D54DDFDD8FE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BC47EE6-B461-423D-AC4B-D3BF6C80663A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D10FEF80-C28A-4A72-8313-80CC4C6A9ADC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40A6276C-A338-4B50-91F6-75A22A686997}"/>
 </file>
</xml_diff>